<commit_message>
auth ve mail update
</commit_message>
<xml_diff>
--- a/storage/uploads/sablon.xlsx
+++ b/storage/uploads/sablon.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fairteknoloji-my.sharepoint.com/personal/batuhan_aytac_fairteknoloji_com_tr/Documents/Masaüstü/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_17DA8375632F8E1ED8920972EDA4D34313025017" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0D77F10-2261-47BB-8B2D-A68E3448BFAC}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_17DA8375632F8E1ED8920972EDA4D34313025017" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{159614FD-9331-4BE2-8D7B-2708E45488CF}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,10 +40,10 @@
     <t>Batuhan Arman Aytaç</t>
   </si>
   <si>
-    <t>batuhanaytac37@gmail.com</t>
-  </si>
-  <si>
     <t>bilişim</t>
+  </si>
+  <si>
+    <t>batuhanarmnx@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -133,6 +133,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -447,10 +451,10 @@
         <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>